<commit_message>
updated org risk assessment
</commit_message>
<xml_diff>
--- a/src/main/resources/RiskAssessment_Field_Values.xlsx
+++ b/src/main/resources/RiskAssessment_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFD56B0-64DA-4CF7-874C-7D17944B52A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF1073E-B2FF-4B6F-8DCF-A080231A98D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="150" yWindow="45" windowWidth="20355" windowHeight="10920" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="45" windowWidth="20355" windowHeight="10920" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RiskAssessmentValues2" sheetId="1" r:id="rId1"/>

</xml_diff>